<commit_message>
client: "Phổ Công" -> "Đánh thường" trên mọi mặt; script deploy từ PC (tools/deploy-haitac.sh)
- chuan-hoa-dich.py: thêm 普攻 "phổ công" -> "đánh thường" vào GLOSSARY (giữ hoa/thường). Áp cho
  templates.bin (104 ô: 49 tên đòn thường trong 文本库, 52 tên/mô tả buff, 3 mô tả vật phẩm)
  -> res/97cec-0a229-5f56f, manifest trỏ theo; excel-src 652 ô (combat, hero, hero-summon,
  text-localization) -> 4 workbook biên dịch lại.
- tools/deploy-haitac.sh: push, scp res mới theo manifest, git pull + up -d --build nginx php trên
  157.66.218.20 (tự kèm docker-compose.domain.yml), --excel copy Excel vào container game + restart.
  Host haitac / khoá ~/.ssh/haitac trên PC; khoá còn phải cài vào authorized_keys của máy chủ.
- docs/ra-soat-chu-client.md, CLAUDE.md mục 9/15 cập nhật.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/excel/release/hero-summon.xlsx
+++ b/server/excel/release/hero-summon.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="英雄召唤" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="英雄召唤星组" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="英雄召唤作弊" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sheet(基础召唤概率)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sheet(友情召唤概率)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sheet(高级召唤概率)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sheet(积分召唤概率)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="英雄召唤" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="英雄召唤星组" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="英雄召唤作弊" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet(基础召唤概率)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet(友情召唤概率)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet(高级召唤概率)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet(积分召唤概率)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -698,7 +698,7 @@
     <t xml:space="preserve">修正</t>
   </si>
   <si>
-    <t xml:space="preserve">Phổ Công</t>
+    <t xml:space="preserve">Đánh thường</t>
   </si>
   <si>
     <t xml:space="preserve">Y Sư</t>

</xml_diff>